<commit_message>
LMDI: Merge pull request #54 from folkehelseinstituttet/fix/fsh-kvalitetsrydding
Retter feil og inkonsistenser i FSH-profiler 8016f72c248c2c01f47fd8b0b518a9ee9e993594
</commit_message>
<xml_diff>
--- a/currentbuild/StructureDefinition-lmdi-del-av-behandlingsregime.xlsx
+++ b/currentbuild/StructureDefinition-lmdi-del-av-behandlingsregime.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-11T12:27:06+00:00</t>
+    <t>2026-03-11T13:36:16+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -132,7 +132,7 @@
     <t>Context</t>
   </si>
   <si>
-    <t>element:Element</t>
+    <t>element:MedicationRequest</t>
   </si>
   <si>
     <t>ID</t>

</xml_diff>